<commit_message>
feat(itrust-study): publish specification and test suite v6.0
</commit_message>
<xml_diff>
--- a/output/xlsx/UC7OfficeVisit--GT-.xlsx
+++ b/output/xlsx/UC7OfficeVisit--GT-.xlsx
@@ -29,7 +29,7 @@
     <t xml:space="preserve">Version: </t>
   </si>
   <si>
-    <t>4.0</t>
+    <t>6.0</t>
   </si>
   <si>
     <t>Suite Type:</t>
@@ -122,7 +122,7 @@
     <t>Alternative Flow 2: Provide additional details about the</t>
   </si>
   <si>
-    <t>hcp: The HCP provides additional details about the office visit as appropriate for the appointment type: General Checkup Basic Health Metrics (uc8)</t>
+    <t>hcp: The HCP provides additional details about the office visit as appropriate for the appointment type: General Checkup Basic Health Metrics (uc8) [Ophthalmology Office Visit](uc21) [Ophthalmology Surgeries](uc22)</t>
   </si>
   <si>
     <t>TC4</t>

</xml_diff>